<commit_message>
Enhanced YOLOv5 with Ghost modules, MoE architecture, and comprehensive analysis tools
- Added Ghost module implementations for efficient model architecture
- Implemented Mixture of Experts (MoE) with sparse and hybrid variants
- Added Squeeze-and-Excitation (SE) attention mechanism
- Enhanced model analysis tools with activation parameter calculations
- Added comprehensive prediction analysis and error evaluation
- Implemented focal loss and knowledge distillation experiments
- Added weighted feature fusion (WFF) capabilities
- Enhanced early stopping with smooth averaging
- Added extensive documentation and guides in GUIDE/ directory
- Implemented VAE-based data augmentation tools
- Added safety compliance analysis and hierarchical evaluation
- Enhanced training scripts with multiple model variants
- Added paper documentation and LaTeX templates
- Comprehensive code reorganization and cleanup

Note: Large training weights and datasets excluded to reduce repository size
</commit_message>
<xml_diff>
--- a/runs/train200epoch/模型分析汇总.xlsx
+++ b/runs/train200epoch/模型分析汇总.xlsx
@@ -493,10 +493,10 @@
         <v>4.8</v>
       </c>
       <c r="F2" t="n">
-        <v>1.59</v>
+        <v>1.73</v>
       </c>
       <c r="G2" t="n">
-        <v>627.7</v>
+        <v>577.5</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -527,10 +527,10 @@
         <v>4.8</v>
       </c>
       <c r="F3" t="n">
-        <v>2.4</v>
+        <v>2.63</v>
       </c>
       <c r="G3" t="n">
-        <v>416.2</v>
+        <v>379.8</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -561,10 +561,10 @@
         <v>7.3</v>
       </c>
       <c r="F4" t="n">
-        <v>1.3</v>
+        <v>1.37</v>
       </c>
       <c r="G4" t="n">
-        <v>768.9</v>
+        <v>730.4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -595,10 +595,10 @@
         <v>7.4</v>
       </c>
       <c r="F5" t="n">
-        <v>2.21</v>
+        <v>2.27</v>
       </c>
       <c r="G5" t="n">
-        <v>453.4</v>
+        <v>439.7</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -629,10 +629,10 @@
         <v>7.3</v>
       </c>
       <c r="F6" t="n">
-        <v>1.28</v>
+        <v>1.38</v>
       </c>
       <c r="G6" t="n">
-        <v>780.2</v>
+        <v>726</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>

</xml_diff>